<commit_message>
Uploaded the updated notebooks and customers EDA file
</commit_message>
<xml_diff>
--- a/EDA/AML_Dataset_Summary.xlsx
+++ b/EDA/AML_Dataset_Summary.xlsx
@@ -568,10 +568,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>8500</v>
+        <v>4500</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>6</v>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>8500</v>
+        <v>4500</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>ACCOUNTS — Total Records: 8,500</t>
+          <t>ACCOUNTS — Total Records: 4,500</t>
         </is>
       </c>
     </row>
@@ -945,10 +945,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2470</v>
+        <v>1298</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>29.06</v>
+        <v>28.84</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -956,10 +956,10 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>5060</v>
+        <v>2602</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>59.53</v>
+        <v>57.82</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="J5" s="5" t="n">
-        <v>8500</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="6">
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1275</v>
+        <v>716</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>15</v>
+        <v>15.91</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -988,10 +988,10 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2557</v>
+        <v>1371</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>30.08</v>
+        <v>30.47</v>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>36123.35</v>
+        <v>36278.61</v>
       </c>
     </row>
     <row r="7">
@@ -1009,10 +1009,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1092</v>
+        <v>573</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>12.85</v>
+        <v>12.73</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
@@ -1020,10 +1020,10 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>883</v>
+        <v>527</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>10.39</v>
+        <v>11.71</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -1031,20 +1031,20 @@
         </is>
       </c>
       <c r="J7" s="5" t="n">
-        <v>44608.44</v>
+        <v>48062.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>retired</t>
+          <t>government_employee</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>949</v>
+        <v>487</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>11.16</v>
+        <v>10.82</v>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
@@ -1052,20 +1052,20 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>527.49</v>
+        <v>643.67</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>government_employee</t>
+          <t>retired</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>873</v>
+        <v>459</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>10.27</v>
+        <v>10.2</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
@@ -1073,20 +1073,20 @@
         </is>
       </c>
       <c r="J9" s="5" t="n">
-        <v>11165.28</v>
+        <v>10868.94</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>freelancer</t>
+          <t>student</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>653</v>
+        <v>363</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>7.68</v>
+        <v>8.07</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1099,20 +1099,20 @@
         </is>
       </c>
       <c r="J10" s="7" t="n">
-        <v>21793.16</v>
+        <v>21735.51</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>student</t>
+          <t>freelancer</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>609</v>
+        <v>305</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>7.16</v>
+        <v>6.78</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="J11" s="5" t="n">
-        <v>43394.32</v>
+        <v>43940.85</v>
       </c>
     </row>
     <row r="12">
@@ -1145,10 +1145,10 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>579</v>
+        <v>299</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>6.81</v>
+        <v>6.64</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -1156,10 +1156,10 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>4282</v>
+        <v>2184</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>50.38</v>
+        <v>48.53</v>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J12" s="7" t="n">
-        <v>594079.71</v>
+        <v>883480.5</v>
       </c>
     </row>
     <row r="13">
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>2604</v>
+        <v>1413</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>30.64</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="14">
@@ -1190,10 +1190,10 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>1614</v>
+        <v>903</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>18.99</v>
+        <v>20.07</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1242,10 +1242,10 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>2926</v>
+        <v>1566</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>34.42</v>
+        <v>34.8</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="J17" s="5" t="n">
-        <v>8500</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="18">
@@ -1268,10 +1268,10 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>2237</v>
+        <v>1143</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>26.32</v>
+        <v>25.4</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1005.82</v>
+        <v>1013.68</v>
       </c>
     </row>
     <row r="19">
@@ -1304,10 +1304,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>1286</v>
+        <v>682</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>15.13</v>
+        <v>15.16</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1065</v>
+        <v>593</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>12.53</v>
+        <v>13.18</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="J19" s="5" t="n">
-        <v>566.0599999999999</v>
+        <v>574.23</v>
       </c>
     </row>
     <row r="20">
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>1185</v>
+        <v>643</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>13.94</v>
+        <v>14.29</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>1045</v>
+        <v>586</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>12.29</v>
+        <v>13.02</v>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
@@ -1368,10 +1368,10 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>866</v>
+        <v>466</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>10.19</v>
+        <v>10.36</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -1379,10 +1379,10 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>971</v>
+        <v>555</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>11.42</v>
+        <v>12.33</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
@@ -1390,20 +1390,20 @@
         </is>
       </c>
       <c r="J21" s="5" t="n">
-        <v>520</v>
+        <v>507.75</v>
       </c>
     </row>
     <row r="22">
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>real_estate</t>
+          <t>healthcare</t>
         </is>
       </c>
       <c r="F22" s="7" t="n">
-        <v>844</v>
+        <v>469</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.93</v>
+        <v>10.42</v>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>996</v>
+        <v>1022.5</v>
       </c>
     </row>
     <row r="23">
@@ -1421,10 +1421,10 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>841</v>
+        <v>435</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>9.890000000000001</v>
+        <v>9.67</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="J23" s="5" t="n">
-        <v>1494.25</v>
+        <v>1508.25</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -1443,14 +1443,14 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>healthcare</t>
+          <t>real_estate</t>
         </is>
       </c>
       <c r="F24" s="7" t="n">
-        <v>839</v>
+        <v>414</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>9.869999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
@@ -1479,14 +1479,14 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>education</t>
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>788</v>
+        <v>385</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>9.27</v>
+        <v>8.56</v>
       </c>
     </row>
     <row r="26">
@@ -1496,21 +1496,21 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4255</v>
+        <v>2203</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>50.06</v>
+        <v>48.96</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="F26" s="7" t="n">
-        <v>779</v>
+        <v>371</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>9.16</v>
+        <v>8.24</v>
       </c>
     </row>
     <row r="27">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>2529</v>
+        <v>1317</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>29.75</v>
+        <v>29.27</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -1531,10 +1531,10 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>702</v>
+        <v>346</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>8.26</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="28">
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1716</v>
+        <v>980</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>20.19</v>
+        <v>21.78</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
@@ -1555,10 +1555,10 @@
         </is>
       </c>
       <c r="F28" s="7" t="n">
-        <v>626</v>
+        <v>346</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>7.36</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -1612,10 +1612,10 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>4347</v>
+        <v>2195</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>51.14</v>
+        <v>48.78</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -1636,10 +1636,10 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>2479</v>
+        <v>1398</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>29.16</v>
+        <v>31.07</v>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>1267</v>
+        <v>698</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>14.91</v>
+        <v>15.51</v>
       </c>
     </row>
     <row r="36">
@@ -1673,10 +1673,10 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>407</v>
+        <v>209</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>4.79</v>
+        <v>4.64</v>
       </c>
     </row>
   </sheetData>
@@ -1719,7 +1719,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERS — Total Records: 5,000</t>
+          <t>CUSTOMERS — Total Records: 3,000</t>
         </is>
       </c>
     </row>
@@ -1789,10 +1789,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1463</v>
+        <v>888</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>29.26</v>
+        <v>29.6</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -1800,10 +1800,10 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>3016</v>
+        <v>1770</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>60.32</v>
+        <v>59</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="J5" s="5" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="6">
@@ -1821,10 +1821,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>741</v>
+        <v>464</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>14.82</v>
+        <v>15.47</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -1832,10 +1832,10 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1467</v>
+        <v>911</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>29.34</v>
+        <v>30.37</v>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>45.23</v>
+        <v>45.11</v>
       </c>
     </row>
     <row r="7">
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>639</v>
+        <v>362</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>12.78</v>
+        <v>12.07</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>517</v>
+        <v>319</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>10.34</v>
+        <v>10.63</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -1875,20 +1875,20 @@
         </is>
       </c>
       <c r="J7" s="5" t="n">
-        <v>14.14</v>
+        <v>14.06</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>government_employee</t>
+          <t>retired</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>516</v>
+        <v>318</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>10.32</v>
+        <v>10.6</v>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
@@ -1902,14 +1902,14 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>retired</t>
+          <t>government_employee</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>500</v>
+        <v>317</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>10</v>
+        <v>10.57</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
@@ -1923,14 +1923,14 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>freelancer</t>
+          <t>student</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>409</v>
+        <v>237</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>8.18</v>
+        <v>7.9</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1949,14 +1949,14 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>student</t>
+          <t>unemployed</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>384</v>
+        <v>214</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>7.68</v>
+        <v>7.13</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -1985,14 +1985,14 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>unemployed</t>
+          <t>freelancer</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>348</v>
+        <v>200</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>6.96</v>
+        <v>6.67</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
@@ -2000,10 +2000,10 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2494</v>
+        <v>1485</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>49.88</v>
+        <v>49.5</v>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
@@ -2021,10 +2021,10 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>1522</v>
+        <v>913</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>30.44</v>
+        <v>30.43</v>
       </c>
     </row>
     <row r="14">
@@ -2034,10 +2034,10 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>984</v>
+        <v>602</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>19.68</v>
+        <v>20.07</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -2086,10 +2086,10 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1775</v>
+        <v>1036</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>35.5</v>
+        <v>34.53</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
         </is>
       </c>
       <c r="J17" s="5" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="18">
@@ -2112,10 +2112,10 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>1287</v>
+        <v>776</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>25.74</v>
+        <v>25.87</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1835.78</v>
+        <v>1838.4</v>
       </c>
     </row>
     <row r="19">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>750</v>
+        <v>467</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>15</v>
+        <v>15.57</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -2159,10 +2159,10 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>657</v>
+        <v>407</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>13.14</v>
+        <v>13.57</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="J19" s="5" t="n">
-        <v>1055.56</v>
+        <v>1036.87</v>
       </c>
     </row>
     <row r="20">
@@ -2180,10 +2180,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>704</v>
+        <v>418</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>14.08</v>
+        <v>13.93</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
@@ -2191,10 +2191,10 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>621</v>
+        <v>386</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>12.42</v>
+        <v>12.87</v>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
@@ -2212,10 +2212,10 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>484</v>
+        <v>303</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>9.68</v>
+        <v>10.1</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -2223,10 +2223,10 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>575</v>
+        <v>362</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>11.5</v>
+        <v>12.07</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
@@ -2234,20 +2234,20 @@
         </is>
       </c>
       <c r="J21" s="5" t="n">
-        <v>910</v>
+        <v>942.75</v>
       </c>
     </row>
     <row r="22">
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>healthcare</t>
         </is>
       </c>
       <c r="F22" s="7" t="n">
-        <v>497</v>
+        <v>304</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.94</v>
+        <v>10.13</v>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
@@ -2255,20 +2255,20 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1830</v>
+        <v>1842.5</v>
       </c>
     </row>
     <row r="23">
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>healthcare</t>
+          <t>real_estate</t>
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>492</v>
+        <v>282</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>9.84</v>
+        <v>9.4</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="J23" s="5" t="n">
-        <v>2763</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -2287,14 +2287,14 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="F24" s="7" t="n">
-        <v>489</v>
+        <v>279</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>9.779999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
@@ -2327,10 +2327,10 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>448</v>
+        <v>264</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>8.960000000000001</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -2340,21 +2340,21 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2548</v>
+        <v>1490</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>50.96</v>
+        <v>49.67</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>real_estate</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="F26" s="7" t="n">
-        <v>446</v>
+        <v>255</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>8.92</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="27">
@@ -2364,21 +2364,21 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>1462</v>
+        <v>869</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>29.24</v>
+        <v>28.97</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>hospitality</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>403</v>
+        <v>232</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>8.06</v>
+        <v>7.73</v>
       </c>
     </row>
     <row r="28">
@@ -2388,21 +2388,21 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>990</v>
+        <v>641</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>19.8</v>
+        <v>21.37</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>hospitality</t>
         </is>
       </c>
       <c r="F28" s="7" t="n">
-        <v>372</v>
+        <v>229</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>7.44</v>
+        <v>7.63</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -2456,10 +2456,10 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>2566</v>
+        <v>1480</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>51.32</v>
+        <v>49.33</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -2480,10 +2480,10 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>1449</v>
+        <v>923</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>28.98</v>
+        <v>30.77</v>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
@@ -2504,10 +2504,10 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>754</v>
+        <v>468</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>15.08</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="36">
@@ -2517,10 +2517,10 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>231</v>
+        <v>129</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>4.62</v>
+        <v>4.3</v>
       </c>
     </row>
   </sheetData>
@@ -2547,7 +2547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2558,7 +2558,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>BENEFICIARIES — Total Records: 6,000</t>
+          <t>BENEFICIARIES — Total Records: 4,000</t>
         </is>
       </c>
     </row>
@@ -2593,36 +2593,36 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3632</v>
+        <v>2216</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>60.53</v>
+        <v>55.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>merchant</t>
+          <t>business</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1787</v>
+        <v>995</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>29.78</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>offshore</t>
+          <t>shell_company</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>296</v>
+        <v>355</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>4.93</v>
+        <v>8.880000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -2632,162 +2632,175 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>285</v>
+        <v>252</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.75</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>4.55</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Beneficiary Country Risk</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Country Risk</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Percentage (%)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
-        <v>3940</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>65.67</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="n">
+        <v>2193</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>54.82</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>1481</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>24.68</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="n">
+        <v>1054</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>26.35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>579</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>9.65</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="B16" s="5" t="n">
+        <v>753</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>18.82</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Risk Commentary by Type</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Risk Commentary</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>individual</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>60.8%</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Standard personal transfers — baseline risk</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>merchant</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>30.2%</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Business/retail transactions — moderate risk</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>offshore</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>4.6%</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>⚠️ Offshore entities — elevated AML risk</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>crypto</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>4.4%</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>🔴 Crypto wallets — high anonymity, high AML concern</t>
         </is>
@@ -2795,10 +2808,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A18:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2826,7 +2839,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>DEVICES — Total Records: 4,500</t>
+          <t>DEVICES — Total Records: 4,000</t>
         </is>
       </c>
     </row>
@@ -2876,10 +2889,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1994</v>
+        <v>1748</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>44.31</v>
+        <v>43.7</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -2887,7 +2900,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>4500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="6">
@@ -2897,10 +2910,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1860</v>
+        <v>1649</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>41.33</v>
+        <v>41.22</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -2908,7 +2921,7 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>778.26</v>
+        <v>764.59</v>
       </c>
     </row>
     <row r="7">
@@ -2918,10 +2931,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>448</v>
+        <v>418</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>9.960000000000001</v>
+        <v>10.45</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2942,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>420.1</v>
+        <v>428.81</v>
       </c>
     </row>
     <row r="8">
@@ -2939,10 +2952,10 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.4</v>
+        <v>4.62</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
@@ -2960,7 +2973,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>422</v>
+        <v>386</v>
       </c>
     </row>
     <row r="10">
@@ -2970,7 +2983,7 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>786</v>
+        <v>766.5</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -2985,7 +2998,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1151</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="12">
@@ -3020,10 +3033,10 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>4299</v>
+        <v>3807</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>95.53</v>
+        <v>95.18000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -3033,10 +3046,10 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>4.47</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -3085,10 +3098,10 @@
         </is>
       </c>
       <c r="F17" s="5" t="n">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>4.47</v>
+        <v>4.82</v>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
@@ -3123,10 +3136,10 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>374</v>
+        <v>305</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>8.31</v>
+        <v>7.62</v>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
@@ -3146,10 +3159,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4126</v>
+        <v>3695</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>91.69</v>
+        <v>92.38</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -3157,10 +3170,10 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>2.84</v>
+        <v>2.82</v>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
@@ -3180,10 +3193,10 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>374</v>
+        <v>305</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>8.31</v>
+        <v>7.62</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
@@ -3191,10 +3204,10 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>4.4</v>
+        <v>4.62</v>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
@@ -3238,10 +3251,10 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>4372</v>
+        <v>3887</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>97.16</v>
+        <v>97.18000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -3251,10 +3264,10 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2.84</v>
+        <v>2.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>